<commit_message>
Daily NSE scan: 2026-09-30
</commit_message>
<xml_diff>
--- a/output/2026-09-30/enriched_analysis.xlsx
+++ b/output/2026-09-30/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.313</v>
+        <v>3.314</v>
       </c>
       <c r="W2" t="n">
-        <v>2898</v>
+        <v>2897</v>
       </c>
       <c r="X2" t="n">
         <v>22.7</v>
@@ -1164,7 +1164,7 @@
         <v>0.05</v>
       </c>
       <c r="W3" t="n">
-        <v>2676</v>
+        <v>2677</v>
       </c>
       <c r="X3" t="n">
         <v>9.199999999999999</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.923</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="W4" t="n">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="X4" t="n">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="Y4" t="n">
         <v>22</v>
@@ -1553,16 +1553,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Signet Industries Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1570,10 +1570,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G5" t="n">
         <v>17</v>
@@ -1582,28 +1582,28 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>68.37</v>
+        <v>5204.5</v>
       </c>
       <c r="J5" t="n">
-        <v>74.22</v>
+        <v>5198.76</v>
       </c>
       <c r="K5" t="n">
-        <v>-7.9</v>
+        <v>0.1</v>
       </c>
       <c r="L5" t="n">
-        <v>72.56999999999999</v>
+        <v>67.16</v>
       </c>
       <c r="M5" t="n">
-        <v>2.01</v>
+        <v>7.21</v>
       </c>
       <c r="N5" t="n">
-        <v>20066329</v>
+        <v>72054758</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>20066329</v>
+        <v>72054758</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -1617,60 +1617,60 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.003</v>
+        <v>0.045</v>
       </c>
       <c r="W5" t="n">
-        <v>200</v>
+        <v>16177</v>
       </c>
       <c r="X5" t="n">
-        <v>8.48</v>
+        <v>41.2</v>
       </c>
       <c r="Y5" t="n">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="Z5" t="n">
-        <v>27.97</v>
+        <v>145</v>
       </c>
       <c r="AA5" t="n">
-        <v>17</v>
+        <v>264</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.73</v>
+        <v>27.38</v>
       </c>
       <c r="AC5" t="n">
-        <v>13.6</v>
+        <v>25.5</v>
       </c>
       <c r="AD5" t="n">
-        <v>1.86</v>
+        <v>0.64</v>
       </c>
       <c r="AE5" t="b">
         <v>1</v>
       </c>
       <c r="AF5" t="n">
-        <v>9.140000000000001</v>
+        <v>5</v>
       </c>
       <c r="AG5" t="n">
-        <v>65.04000000000001</v>
+        <v>5463.92</v>
       </c>
       <c r="AH5" t="n">
-        <v>53.06</v>
+        <v>4475.56</v>
       </c>
       <c r="AI5" t="n">
-        <v>49.1</v>
+        <v>44.6</v>
       </c>
       <c r="AJ5" t="n">
-        <v>74.21830535305453</v>
+        <v>5198.755988455989</v>
       </c>
       <c r="AK5" t="n">
-        <v>-7.9</v>
+        <v>0.1</v>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
@@ -1689,52 +1689,52 @@
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>04-08-2026</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="AQ5" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="AR5" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="AS5" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="AT5" t="n">
         <v>0</v>
       </c>
       <c r="AU5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV5" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AW5" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="AX5" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="AY5" t="n">
         <v>0</v>
       </c>
       <c r="AZ5" t="n">
-        <v>1525105</v>
+        <v>0</v>
       </c>
       <c r="BA5" t="n">
-        <v>9663835</v>
+        <v>0</v>
       </c>
       <c r="BB5" t="n">
-        <v>20066329</v>
+        <v>72054758</v>
       </c>
       <c r="BC5" t="n">
-        <v>20066329</v>
+        <v>72054758</v>
       </c>
       <c r="BD5" t="n">
         <v>0</v>
@@ -1770,10 +1770,10 @@
         <v>0</v>
       </c>
       <c r="BO5" t="n">
-        <v>9663835</v>
+        <v>0</v>
       </c>
       <c r="BP5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ5" t="n">
         <v>0</v>
@@ -1785,12 +1785,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1802,107 +1802,107 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="G6" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>575.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>510.94</v>
+      </c>
+      <c r="K6" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="L6" t="n">
+        <v>62.09</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="N6" t="n">
+        <v>30622049</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>30622049</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S6" t="b">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
         <v>17</v>
       </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>5204.5</v>
-      </c>
-      <c r="J6" t="n">
-        <v>5198.76</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>67.16</v>
-      </c>
-      <c r="M6" t="n">
-        <v>7.21</v>
-      </c>
-      <c r="N6" t="n">
-        <v>72054758</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>72054758</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S6" t="b">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>6</v>
-      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0.045</v>
+        <v>0.31</v>
       </c>
       <c r="W6" t="n">
-        <v>16183</v>
+        <v>988</v>
       </c>
       <c r="X6" t="n">
-        <v>41.2</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="Y6" t="n">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="Z6" t="n">
-        <v>145</v>
+        <v>30</v>
       </c>
       <c r="AA6" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>27.38</v>
+        <v>14.66</v>
       </c>
       <c r="AC6" t="n">
-        <v>25.5</v>
+        <v>14.4</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.64</v>
+        <v>0.01</v>
       </c>
       <c r="AE6" t="b">
         <v>1</v>
       </c>
       <c r="AF6" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="AG6" t="n">
-        <v>5463.92</v>
+        <v>509.85</v>
       </c>
       <c r="AH6" t="n">
-        <v>4475.56</v>
+        <v>490.71</v>
       </c>
       <c r="AI6" t="n">
-        <v>44.6</v>
+        <v>34.8</v>
       </c>
       <c r="AJ6" t="n">
-        <v>5198.755988455989</v>
+        <v>510.9380308010612</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.1</v>
+        <v>12.6</v>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
@@ -1916,57 +1916,57 @@
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>04-08-2026</t>
+          <t>26-08-2026</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="AQ6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AR6" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="AS6" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="AT6" t="n">
         <v>0</v>
       </c>
       <c r="AU6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="AW6" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AX6" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="AY6" t="n">
         <v>0</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0</v>
+        <v>9018372</v>
       </c>
       <c r="BA6" t="n">
-        <v>0</v>
+        <v>24967565</v>
       </c>
       <c r="BB6" t="n">
-        <v>72054758</v>
+        <v>30622049</v>
       </c>
       <c r="BC6" t="n">
-        <v>72054758</v>
+        <v>30622049</v>
       </c>
       <c r="BD6" t="n">
         <v>0</v>
@@ -2002,10 +2002,10 @@
         <v>0</v>
       </c>
       <c r="BO6" t="n">
-        <v>0</v>
+        <v>24967565</v>
       </c>
       <c r="BP6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BQ6" t="n">
         <v>0</v>
@@ -2017,16 +2017,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
+          <t>Signet Industries Limited</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -2034,40 +2034,40 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G7" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>575.5</v>
+        <v>68.37</v>
       </c>
       <c r="J7" t="n">
-        <v>510.94</v>
+        <v>74.22</v>
       </c>
       <c r="K7" t="n">
-        <v>12.6</v>
+        <v>-7.9</v>
       </c>
       <c r="L7" t="n">
-        <v>62.09</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>3.06</v>
+        <v>2.01</v>
       </c>
       <c r="N7" t="n">
-        <v>30622049</v>
+        <v>20066329</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>30622049</v>
+        <v>20066329</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -2081,91 +2081,91 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
+        <v>18</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>21-09-2026</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="W7" t="n">
+        <v>201</v>
+      </c>
+      <c r="X7" t="n">
+        <v>8.550000000000001</v>
+      </c>
+      <c r="Y7" t="n">
         <v>17</v>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="Z7" t="n">
+        <v>27.97</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>17</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="AE7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>9.140000000000001</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>65.04000000000001</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>53.06</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>74.21830535305453</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>-7.9</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
         <is>
           <t>21-09-2026</t>
         </is>
       </c>
-      <c r="V7" t="n">
-        <v>0.312</v>
-      </c>
-      <c r="W7" t="n">
-        <v>980</v>
-      </c>
-      <c r="X7" t="n">
-        <v>9.640000000000001</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>30</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>14.66</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AE7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>14</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>509.85</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>490.71</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>510.9380308010612</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>26-08-2026</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>21-09-2026</t>
-        </is>
-      </c>
       <c r="AQ7" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="AR7" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="AS7" t="n">
         <v>9</v>
@@ -2174,31 +2174,31 @@
         <v>0</v>
       </c>
       <c r="AU7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AV7" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="AW7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AX7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AY7" t="n">
         <v>0</v>
       </c>
       <c r="AZ7" t="n">
-        <v>9018372</v>
+        <v>1525105</v>
       </c>
       <c r="BA7" t="n">
-        <v>24967565</v>
+        <v>9663835</v>
       </c>
       <c r="BB7" t="n">
-        <v>30622049</v>
+        <v>20066329</v>
       </c>
       <c r="BC7" t="n">
-        <v>30622049</v>
+        <v>20066329</v>
       </c>
       <c r="BD7" t="n">
         <v>0</v>
@@ -2234,10 +2234,10 @@
         <v>0</v>
       </c>
       <c r="BO7" t="n">
-        <v>24967565</v>
+        <v>9663835</v>
       </c>
       <c r="BP7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ7" t="n">
         <v>0</v>
@@ -2321,10 +2321,10 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.437</v>
+        <v>0.438</v>
       </c>
       <c r="W8" t="n">
-        <v>2787</v>
+        <v>2785</v>
       </c>
       <c r="X8" t="n">
         <v>22.8</v>
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>2.324</v>
+        <v>2.334</v>
       </c>
       <c r="W10" t="n">
-        <v>2526</v>
+        <v>2515</v>
       </c>
       <c r="X10" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Y10" t="n">
         <v>6</v>
@@ -3018,10 +3018,10 @@
         <v>0.13</v>
       </c>
       <c r="W11" t="n">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="X11" t="n">
-        <v>28.8</v>
+        <v>28.7</v>
       </c>
       <c r="Y11" t="n">
         <v>17</v>
@@ -3476,10 +3476,10 @@
         <v>0.05</v>
       </c>
       <c r="W13" t="n">
-        <v>1644</v>
+        <v>1649</v>
       </c>
       <c r="X13" t="n">
-        <v>22.1</v>
+        <v>22.2</v>
       </c>
       <c r="Y13" t="n">
         <v>55</v>
@@ -3705,10 +3705,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>2.852</v>
+        <v>2.86</v>
       </c>
       <c r="W14" t="n">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="X14" t="n">
         <v>25.9</v>
@@ -3934,10 +3934,10 @@
         <v>0.062</v>
       </c>
       <c r="W15" t="n">
-        <v>1777</v>
+        <v>1783</v>
       </c>
       <c r="X15" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="Y15" t="n">
         <v>20</v>
@@ -4163,10 +4163,10 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="W16" t="n">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="X16" t="n">
         <v>11</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="W17" t="n">
-        <v>790</v>
+        <v>803</v>
       </c>
       <c r="X17" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="Y17" t="n">
         <v>19</v>
@@ -4625,13 +4625,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.376</v>
+        <v>0.374</v>
       </c>
       <c r="W18" t="n">
-        <v>1096</v>
+        <v>1104</v>
       </c>
       <c r="X18" t="n">
-        <v>55.8</v>
+        <v>56.2</v>
       </c>
       <c r="Y18" t="n">
         <v>21</v>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.502</v>
+        <v>0.503</v>
       </c>
       <c r="W19" t="n">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="X19" t="n">
-        <v>36.9</v>
+        <v>36.8</v>
       </c>
       <c r="Y19" t="n">
         <v>21</v>
@@ -5092,10 +5092,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W20" t="n">
-        <v>52237</v>
+        <v>52260</v>
       </c>
       <c r="X20" t="n">
-        <v>44.2</v>
+        <v>44.3</v>
       </c>
       <c r="Y20" t="n">
         <v>5</v>
@@ -5321,13 +5321,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.183</v>
+        <v>0.179</v>
       </c>
       <c r="W21" t="n">
-        <v>604</v>
+        <v>619</v>
       </c>
       <c r="X21" t="n">
-        <v>50.5</v>
+        <v>51.8</v>
       </c>
       <c r="Y21" t="n">
         <v>3</v>
@@ -5345,7 +5345,7 @@
         <v>11.6</v>
       </c>
       <c r="AD21" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AE21" t="b">
         <v>1</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.897</v>
+        <v>0.91</v>
       </c>
       <c r="W22" t="n">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="X22" t="n">
-        <v>6.46</v>
+        <v>6.37</v>
       </c>
       <c r="Y22" t="n">
         <v>31</v>
@@ -5781,13 +5781,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.313</v>
+        <v>0.315</v>
       </c>
       <c r="W23" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="X23" t="n">
-        <v>24</v>
+        <v>23.9</v>
       </c>
       <c r="Y23" t="n">
         <v>12</v>
@@ -6013,13 +6013,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.653</v>
+        <v>0.65</v>
       </c>
       <c r="W24" t="n">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="X24" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="Y24" t="n">
         <v>19</v>
@@ -6245,13 +6245,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="W25" t="n">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="X25" t="n">
-        <v>1166</v>
+        <v>1182</v>
       </c>
       <c r="Y25" t="n">
         <v>-61</v>
@@ -6473,13 +6473,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.495</v>
+        <v>0.488</v>
       </c>
       <c r="W26" t="n">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="X26" t="n">
-        <v>37.6</v>
+        <v>38.1</v>
       </c>
       <c r="Y26" t="n">
         <v>-44</v>
@@ -6708,7 +6708,7 @@
         <v>0.075</v>
       </c>
       <c r="W27" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="X27" t="n">
         <v>13</v>
@@ -6935,13 +6935,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.276</v>
+        <v>0.275</v>
       </c>
       <c r="W28" t="n">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="X28" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="Y28" t="n">
         <v>9</v>
@@ -7170,10 +7170,10 @@
         <v>0.051</v>
       </c>
       <c r="W29" t="n">
-        <v>5108</v>
+        <v>5163</v>
       </c>
       <c r="X29" t="n">
-        <v>33.3</v>
+        <v>33.6</v>
       </c>
       <c r="Y29" t="n">
         <v>-25</v>
@@ -7402,7 +7402,7 @@
         <v>0.045</v>
       </c>
       <c r="W30" t="n">
-        <v>1553</v>
+        <v>1557</v>
       </c>
       <c r="X30" t="n">
         <v>20.3</v>
@@ -7631,13 +7631,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.802</v>
+        <v>0.804</v>
       </c>
       <c r="W31" t="n">
-        <v>3940</v>
+        <v>3931</v>
       </c>
       <c r="X31" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="Y31" t="n">
         <v>2</v>
@@ -8093,10 +8093,10 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.227</v>
+        <v>0.226</v>
       </c>
       <c r="W33" t="n">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="X33" t="n">
         <v>13.6</v>
@@ -8325,13 +8325,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.271</v>
+        <v>0.268</v>
       </c>
       <c r="W34" t="n">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="X34" t="n">
-        <v>14.4</v>
+        <v>14.6</v>
       </c>
       <c r="Y34" t="n">
         <v>16</v>
@@ -8789,10 +8789,10 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.23</v>
+        <v>0.229</v>
       </c>
       <c r="W36" t="n">
-        <v>1736</v>
+        <v>1739</v>
       </c>
       <c r="X36" t="n">
         <v>18.4</v>
@@ -9024,7 +9024,7 @@
         <v>0.02</v>
       </c>
       <c r="W37" t="n">
-        <v>9670</v>
+        <v>9672</v>
       </c>
       <c r="X37" t="n">
         <v>12.8</v>
@@ -9479,13 +9479,13 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.363</v>
+        <v>0.359</v>
       </c>
       <c r="W39" t="n">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="X39" t="n">
-        <v>95.40000000000001</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="Y39" t="n">
         <v>246</v>
@@ -9717,7 +9717,7 @@
         <v>1632</v>
       </c>
       <c r="X40" t="n">
-        <v>29.4</v>
+        <v>29.5</v>
       </c>
       <c r="Y40" t="n">
         <v>39</v>
@@ -9946,7 +9946,7 @@
         <v>0.011</v>
       </c>
       <c r="W41" t="n">
-        <v>4148</v>
+        <v>4158</v>
       </c>
       <c r="X41" t="inlineStr"/>
       <c r="Y41" t="n">
@@ -10176,7 +10176,7 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>4921</v>
+        <v>4916</v>
       </c>
       <c r="X42" t="n">
         <v>11.5</v>
@@ -10405,13 +10405,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.106</v>
+        <v>0.104</v>
       </c>
       <c r="W43" t="n">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="X43" t="n">
-        <v>25.8</v>
+        <v>26.3</v>
       </c>
       <c r="Y43" t="n">
         <v>24</v>
@@ -10872,7 +10872,7 @@
         <v>0.075</v>
       </c>
       <c r="W45" t="n">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="X45" t="n">
         <v>13.4</v>
@@ -11104,10 +11104,10 @@
         <v>0.126</v>
       </c>
       <c r="W46" t="n">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="X46" t="n">
-        <v>6.35</v>
+        <v>6.38</v>
       </c>
       <c r="Y46" t="n">
         <v>118</v>
@@ -11332,7 +11332,7 @@
         <v>0.024</v>
       </c>
       <c r="W47" t="n">
-        <v>1012</v>
+        <v>1022</v>
       </c>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="n">
@@ -11562,10 +11562,10 @@
         <v>0.008</v>
       </c>
       <c r="W48" t="n">
-        <v>5363</v>
+        <v>5381</v>
       </c>
       <c r="X48" t="n">
-        <v>9.06</v>
+        <v>9.09</v>
       </c>
       <c r="Y48" t="n">
         <v>43</v>
@@ -11794,10 +11794,10 @@
         <v>0</v>
       </c>
       <c r="W49" t="n">
-        <v>8871</v>
+        <v>8881</v>
       </c>
       <c r="X49" t="n">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="Y49" t="n">
         <v>21</v>
@@ -12026,10 +12026,10 @@
         <v>0</v>
       </c>
       <c r="W50" t="n">
-        <v>3453</v>
+        <v>3449</v>
       </c>
       <c r="X50" t="n">
-        <v>77.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Y50" t="n">
         <v>42</v>
@@ -12255,13 +12255,13 @@
         </is>
       </c>
       <c r="V51" t="n">
-        <v>0.215</v>
+        <v>0.214</v>
       </c>
       <c r="W51" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="X51" t="n">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="Y51" t="n">
         <v>21</v>
@@ -12490,7 +12490,7 @@
         <v>0</v>
       </c>
       <c r="W52" t="n">
-        <v>115240</v>
+        <v>115270</v>
       </c>
       <c r="X52" t="n">
         <v>33.2</v>
@@ -12824,101 +12824,101 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>THANGAMAYL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Signet Industries Limited</t>
+          <t>THANGAMAYIL JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>68.37</v>
+        <v>5204.5</v>
       </c>
       <c r="D5" t="n">
-        <v>74.22</v>
+        <v>5198.76</v>
       </c>
       <c r="E5" t="n">
-        <v>-7.9</v>
+        <v>0.1</v>
       </c>
       <c r="F5" t="n">
-        <v>72.56999999999999</v>
+        <v>67.16</v>
       </c>
       <c r="G5" t="n">
-        <v>2.01</v>
+        <v>7.21</v>
       </c>
       <c r="H5" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>THANGAMAYL</t>
+          <t>SRHHYPOLTD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THANGAMAYIL JEWELLERY LIMITED</t>
+          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5204.5</v>
+        <v>575.5</v>
       </c>
       <c r="D6" t="n">
-        <v>5198.76</v>
+        <v>510.94</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1</v>
+        <v>12.6</v>
       </c>
       <c r="F6" t="n">
-        <v>67.16</v>
+        <v>62.09</v>
       </c>
       <c r="G6" t="n">
-        <v>7.21</v>
+        <v>3.06</v>
       </c>
       <c r="H6" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SRHHYPOLTD</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sree Rayalaseema Hi-Strength Hypo Limited</t>
+          <t>Signet Industries Limited</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>575.5</v>
+        <v>68.37</v>
       </c>
       <c r="D7" t="n">
-        <v>510.94</v>
+        <v>74.22</v>
       </c>
       <c r="E7" t="n">
-        <v>12.6</v>
+        <v>-7.9</v>
       </c>
       <c r="F7" t="n">
-        <v>62.09</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>3.06</v>
+        <v>2.01</v>
       </c>
       <c r="H7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>

</xml_diff>